<commit_message>
xuatben v41: đọc MRZ hộ chiếu (số+quốc tịch+dob+tên), template bỏ dòng chủ tàu/địa chỉ PHL
</commit_message>
<xml_diff>
--- a/xuatben/assets/template.xlsx
+++ b/xuatben/assets/template.xlsx
@@ -34,16 +34,16 @@
     <t>DANH SÁCH HÀNH KHÁCH</t>
   </si>
   <si>
-    <t>Tên tàu thuyền: Phát Hoàng Long ….......</t>
+    <t xml:space="preserve">Tên tàu thuyền: ……………………………..</t>
   </si>
   <si>
     <t>Số đăng ký:……………………..</t>
   </si>
   <si>
-    <t>Tên chủ tàu thuyền: Cty TNHH Phát Hoàng Long Ninh Thuận</t>
+    <t xml:space="preserve"/>
   </si>
   <si>
-    <t>Địa chỉ: Thôn Vĩnh Hy, Xã Vĩnh Hải, Tỉnh Khánh Hòa, Việt Nam</t>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t>Tên thuyền trưởng:………………………………………..</t>

</xml_diff>